<commit_message>
Add drawings from the report, update README
</commit_message>
<xml_diff>
--- a/calculations/HVAC_Calculations.xlsx
+++ b/calculations/HVAC_Calculations.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Building Envelope" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Loads" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distribution Network" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pump Head" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heat Generator" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chimney Sizing" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Building Envelope" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Total Loads" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Distribution Network" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pump Head" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Heat Generator" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Chimney Sizing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Sources" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -531,7 +531,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -553,7 +552,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -568,7 +566,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -625,7 +622,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -840,7 +836,6 @@
         <v>4.023</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -910,7 +905,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
@@ -1671,7 +1665,6 @@
         <v>504.8</v>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
@@ -1721,7 +1714,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
@@ -2547,7 +2539,6 @@
         <v>425.8</v>
       </c>
     </row>
-    <row r="82"/>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
@@ -2597,7 +2588,6 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
@@ -2699,7 +2689,6 @@
       </c>
       <c r="C93" s="8" t="n"/>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
@@ -2842,7 +2831,6 @@
         <v>3.3408</v>
       </c>
     </row>
-    <row r="103"/>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
@@ -2882,7 +2870,6 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
@@ -3160,7 +3147,6 @@
         <v>2102.4</v>
       </c>
     </row>
-    <row r="124"/>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
@@ -3230,7 +3216,6 @@
         </is>
       </c>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
@@ -3508,7 +3493,6 @@
         <v>1648</v>
       </c>
     </row>
-    <row r="146"/>
     <row r="147">
       <c r="A147" s="5" t="inlineStr">
         <is>
@@ -3578,7 +3562,6 @@
         </is>
       </c>
     </row>
-    <row r="151"/>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
         <is>
@@ -4548,7 +4531,6 @@
         <v>250</v>
       </c>
     </row>
-    <row r="186"/>
     <row r="187">
       <c r="A187" s="5" t="inlineStr">
         <is>
@@ -5831,7 +5813,6 @@
         <v>329276</v>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
@@ -6072,7 +6053,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -6195,7 +6175,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -8307,7 +8286,6 @@
         <v>214163</v>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
@@ -8922,7 +8900,6 @@
         <v>22830.4</v>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
@@ -9052,7 +9029,6 @@
         <v>475.7</v>
       </c>
     </row>
-    <row r="70"/>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
@@ -9220,7 +9196,6 @@
         <v>243686.2</v>
       </c>
     </row>
-    <row r="80"/>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
@@ -9606,7 +9581,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -9889,7 +9863,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -10008,7 +9981,6 @@
       </c>
       <c r="C21" s="8" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
@@ -10114,7 +10086,6 @@
       </c>
       <c r="C29" s="8" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -10295,7 +10266,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -10352,7 +10322,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -10388,7 +10357,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>

</xml_diff>